<commit_message>
chore: rename file and fix typos in content
</commit_message>
<xml_diff>
--- a/data/ProjectMaturityAssessmentReviewTemplate.xlsx
+++ b/data/ProjectMaturityAssessmentReviewTemplate.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5A901B6-DFDB-4FE4-AC62-C796785E581A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EE003AA-02EF-4B20-9201-346F02403F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -336,9 +336,6 @@
     <t>Bugfixing Strategy</t>
   </si>
   <si>
-    <t>Define a strategy for handling bugs during release preparation and in production. This should include the versioning scheme for bugfixes (buildmanagement). Test your strategy with dummy bugs before going into production.</t>
-  </si>
-  <si>
     <t>Bugfixing processes, builds and deployments need to be in place before first production deployment to allow fast reaction when the first bugs are encountered.</t>
   </si>
   <si>
@@ -481,10 +478,6 @@
     <t>Appropriate level of Test automation</t>
   </si>
   <si>
-    <t xml:space="preserve">To get faster results and increase efficiency we use automated test cases where technically and economically possible.
-Agile Integration: We create and execute automated test cases within the same sprint cycle wherever possible to achieve highest efficency. </t>
-  </si>
-  <si>
     <t>Stable test environment and test data</t>
   </si>
   <si>
@@ -501,9 +494,6 @@
 Not only the technical test team should be able to maintain automated tests. By using the right approach members of the functional test can easily maintain the test cases themselves.</t>
   </si>
   <si>
-    <t>Reliability and Reproducability</t>
-  </si>
-  <si>
     <t>Test cases have to be designed in a way they could be reproduced under consistent conditions and deliver identical results.</t>
   </si>
   <si>
@@ -558,9 +548,6 @@
     <t>Business continuity must be planned in the design phase. Discuss availability demand with business</t>
   </si>
   <si>
-    <t>In order to supply robust and stable IT services we need to discuss disaster scenarios and mitigations with the business</t>
-  </si>
-  <si>
     <t>G01</t>
   </si>
   <si>
@@ -615,9 +602,6 @@
     <t>Build results must be stored in a separate repository. Dependent projects and deployments must take the artifacts solely from that repository. This must be done using an appropriate dependency management mechanism of the build system.</t>
   </si>
   <si>
-    <t>Coupling two projects via source code control introduces tracability problems, especially considering tagging and branching. Also it unecessarily increases the buildtime.</t>
-  </si>
-  <si>
     <t>Versioning Scheme</t>
   </si>
   <si>
@@ -670,9 +654,6 @@
   </si>
   <si>
     <t>G-Operations and Support</t>
-  </si>
-  <si>
-    <t>H-Buildmanagement</t>
   </si>
   <si>
     <t>Current (0-5)</t>
@@ -874,12 +855,6 @@
   <si>
     <t>Every commit should be tested as early, thorough and fast as possible. This should be staged by priorities. (Compilability, unit tests, integration tests, code quality)
 A CI build job checks code for buildability and derives immediate feedback to the team about the outcome of the build and quality check.</t>
-  </si>
-  <si>
-    <t>Commits should not be allowed into master branch without passing the defined quality gates. These quality gates must be continuosly adjusted.</t>
-  </si>
-  <si>
-    <t>This allows quick turnaround times for developers using unstable version on actual environments, while minimizing the risk of accidental deployment of those unstable versions to higher environments (including production)</t>
   </si>
   <si>
     <t>Retrospective</t>
@@ -949,12 +924,6 @@
     <t>Unstable test environments and data could increase the effort and lead to wrong results. For functional test and technical tests, test data management is an important prerequisite to ensure reasonable test results.</t>
   </si>
   <si>
-    <t>Tests that are atomic, specific, precise and independent could provide fast feedback on the test result of different features/system functionalities for quick corrective action without the need to isolate the rootcause via human intervention. If test cases are interdependent and tighly coupled, a defect related to the test case in the earlier sequence could block the execution of dependent test cases in later sequence.  Like wise, early test steps that are failed in a long test case could also block the execution of subsequent steps, hence masking the defects could have uncovered by short and atomic tests.</t>
-  </si>
-  <si>
-    <t>This principle is important in order to reduce risk in operation of human errors and imcompliance. This is to ensure that we have stable and performant IT services for our customers.</t>
-  </si>
-  <si>
     <t>Support team needs good analysis options to solve incidents quickly to restore the ITservice as quickly as possible.</t>
   </si>
   <si>
@@ -963,6 +932,37 @@
 •Frequent builds ensure early feedback for timely corrective action if source code breaks
 Ideally, gated check-ins are used (i.e. source code cannot be checked in until builds succeed).
 The later problems are detected, the harder the problems to be fixed. Using an early CI build ensures a minimal quality standard for centralized code repository.</t>
+  </si>
+  <si>
+    <t>This allows quick turnaround times for developers using unstable version on actual environments, while minimizing the risk of accidental deployment of those unstable versions to higher environments (including production).</t>
+  </si>
+  <si>
+    <t>Tests that are atomic, specific, precise and independent could provide fast feedback on the test result of different features/system functionalities for quick corrective action without the need to isolate the rootcause via human intervention. If test cases are interdependent and tightly coupled, a defect related to the test case in the earlier sequence could block the execution of dependent test cases in later sequence.  Like wise, early test steps that are failed in a long test case could also block the execution of subsequent steps, hence masking the defects could have uncovered by short and atomic tests.</t>
+  </si>
+  <si>
+    <t>Coupling two projects via source code control introduces tracability problems, especially considering tagging and branching. Also it unnecessarily increases the build time.</t>
+  </si>
+  <si>
+    <t>Commits should not be allowed into master branch without passing the defined quality gates. These quality gates must be continuously adjusted.</t>
+  </si>
+  <si>
+    <t>Define a strategy for handling bugs during release preparation and in production. This should include the versioning scheme for bugfixes (Build Management). Test your strategy with dummy bugs before going into production.</t>
+  </si>
+  <si>
+    <t>H-Build Management</t>
+  </si>
+  <si>
+    <t>This principle is important in order to reduce risk in operation of human errors and noncompliance. This is to ensure that we have stable and performant IT services for our customers.</t>
+  </si>
+  <si>
+    <t>Reliability and Reproducibility</t>
+  </si>
+  <si>
+    <t>To get faster results and increase efficiency we use automated test cases where technically and economically possible.
+Agile Integration: We create and execute automated test cases within the same sprint cycle wherever possible to achieve highest efficiency.</t>
+  </si>
+  <si>
+    <t>In order to supply robust and stable IT services we need to discuss disaster scenarios and mitigations with the business.</t>
   </si>
 </sst>
 </file>
@@ -5479,16 +5479,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="C1" s="17" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="F1" s="17" t="s">
         <v>3</v>
@@ -5508,7 +5508,7 @@
     </row>
     <row r="2" spans="1:10" ht="240" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>52</v>
@@ -5520,7 +5520,7 @@
         <v>36</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="F2" s="14">
         <v>2</v>
@@ -5536,7 +5536,7 @@
     </row>
     <row r="3" spans="1:10" ht="240" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>53</v>
@@ -5548,7 +5548,7 @@
         <v>37</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="F3" s="14">
         <v>2</v>
@@ -5564,7 +5564,7 @@
     </row>
     <row r="4" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>54</v>
@@ -5592,7 +5592,7 @@
     </row>
     <row r="5" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>55</v>
@@ -5620,7 +5620,7 @@
     </row>
     <row r="6" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>56</v>
@@ -5648,7 +5648,7 @@
     </row>
     <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>57</v>
@@ -5676,7 +5676,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>58</v>
@@ -5704,7 +5704,7 @@
     </row>
     <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>59</v>
@@ -5732,7 +5732,7 @@
     </row>
     <row r="10" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>60</v>
@@ -5760,7 +5760,7 @@
     </row>
     <row r="11" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>61</v>
@@ -5788,7 +5788,7 @@
     </row>
     <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>62</v>
@@ -5816,19 +5816,19 @@
     </row>
     <row r="13" spans="1:10" ht="315" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>63</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>51</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="F13" s="14">
         <v>2</v>
@@ -5844,7 +5844,7 @@
     </row>
     <row r="14" spans="1:10" ht="165" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B14" s="8" t="s">
         <v>64</v>
@@ -5856,7 +5856,7 @@
         <v>66</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="F14" s="14">
         <v>2</v>
@@ -5872,10 +5872,10 @@
     </row>
     <row r="15" spans="1:10" ht="105" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>67</v>
@@ -5900,10 +5900,10 @@
     </row>
     <row r="16" spans="1:10" ht="135" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>70</v>
@@ -5928,19 +5928,19 @@
     </row>
     <row r="17" spans="1:10" ht="120" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="F17" s="14">
         <v>2</v>
@@ -5956,19 +5956,19 @@
     </row>
     <row r="18" spans="1:10" ht="240" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>73</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="F18" s="14">
         <v>2</v>
@@ -5984,10 +5984,10 @@
     </row>
     <row r="19" spans="1:10" ht="120" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>74</v>
@@ -5996,7 +5996,7 @@
         <v>75</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="F19" s="14">
         <v>2</v>
@@ -6012,10 +6012,10 @@
     </row>
     <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>23</v>
@@ -6024,7 +6024,7 @@
         <v>76</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="F20" s="14">
         <v>2</v>
@@ -6040,19 +6040,19 @@
     </row>
     <row r="21" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>77</v>
       </c>
       <c r="D21" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="E21" s="5" t="s">
         <v>78</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>79</v>
       </c>
       <c r="F21" s="14">
         <v>2</v>
@@ -6068,19 +6068,19 @@
     </row>
     <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="F22" s="14">
         <v>2</v>
@@ -6094,19 +6094,19 @@
     </row>
     <row r="23" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="F23" s="14">
         <v>2</v>
@@ -6120,19 +6120,19 @@
     </row>
     <row r="24" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="F24" s="14">
         <v>2</v>
@@ -6146,19 +6146,19 @@
     </row>
     <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="F25" s="14">
         <v>2</v>
@@ -6172,19 +6172,19 @@
     </row>
     <row r="26" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="F26" s="14">
         <v>2</v>
@@ -6198,19 +6198,19 @@
     </row>
     <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="F27" s="14">
         <v>2</v>
@@ -6224,19 +6224,19 @@
     </row>
     <row r="28" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="F28" s="14">
         <v>2</v>
@@ -6250,19 +6250,19 @@
     </row>
     <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="F29" s="14">
         <v>2</v>
@@ -6276,19 +6276,19 @@
     </row>
     <row r="30" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="F30" s="14">
         <v>2</v>
@@ -6302,19 +6302,19 @@
     </row>
     <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="F31" s="14">
         <v>2</v>
@@ -6328,19 +6328,19 @@
     </row>
     <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="F32" s="14">
         <v>2</v>
@@ -6354,19 +6354,19 @@
     </row>
     <row r="33" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="F33" s="14">
         <v>2</v>
@@ -6380,19 +6380,19 @@
     </row>
     <row r="34" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C34" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="E34" s="5" t="s">
         <v>88</v>
-      </c>
-      <c r="E34" s="5" t="s">
-        <v>89</v>
       </c>
       <c r="F34" s="14">
         <v>2</v>
@@ -6408,19 +6408,19 @@
     </row>
     <row r="35" spans="1:10" ht="135" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="F35" s="14">
         <v>2</v>
@@ -6436,19 +6436,19 @@
     </row>
     <row r="36" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C36" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D36" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="E36" s="5" t="s">
         <v>92</v>
-      </c>
-      <c r="E36" s="5" t="s">
-        <v>93</v>
       </c>
       <c r="F36" s="14">
         <v>2</v>
@@ -6464,19 +6464,19 @@
     </row>
     <row r="37" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C37" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="D37" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="D37" s="5" t="s">
-        <v>95</v>
-      </c>
       <c r="E37" s="5" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="F37" s="14">
         <v>2</v>
@@ -6492,19 +6492,19 @@
     </row>
     <row r="38" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C38" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="D38" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="E38" s="5" t="s">
         <v>97</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>98</v>
       </c>
       <c r="F38" s="14">
         <v>2</v>
@@ -6520,19 +6520,19 @@
     </row>
     <row r="39" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C39" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D39" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D39" s="5" t="s">
-        <v>105</v>
-      </c>
       <c r="E39" s="5" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="F39" s="14">
         <v>2</v>
@@ -6548,19 +6548,19 @@
     </row>
     <row r="40" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C40" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D40" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="E40" s="5" t="s">
         <v>107</v>
-      </c>
-      <c r="E40" s="5" t="s">
-        <v>108</v>
       </c>
       <c r="F40" s="14">
         <v>2</v>
@@ -6576,19 +6576,19 @@
     </row>
     <row r="41" spans="1:10" ht="120" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C41" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D41" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="E41" s="5" t="s">
         <v>110</v>
-      </c>
-      <c r="E41" s="5" t="s">
-        <v>111</v>
       </c>
       <c r="F41" s="14">
         <v>2</v>
@@ -6604,19 +6604,19 @@
     </row>
     <row r="42" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C42" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="D42" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="E42" s="5" t="s">
         <v>113</v>
-      </c>
-      <c r="E42" s="5" t="s">
-        <v>114</v>
       </c>
       <c r="F42" s="14">
         <v>2</v>
@@ -6632,19 +6632,19 @@
     </row>
     <row r="43" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A43" s="11" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="F43" s="14">
         <v>2</v>
@@ -6660,19 +6660,19 @@
     </row>
     <row r="44" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A44" s="11" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B44" s="11" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C44" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="E44" s="5" t="s">
         <v>120</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="E44" s="5" t="s">
-        <v>121</v>
       </c>
       <c r="F44" s="14">
         <v>2</v>
@@ -6688,19 +6688,19 @@
     </row>
     <row r="45" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A45" s="11" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B45" s="11" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="F45" s="14">
         <v>2</v>
@@ -6716,19 +6716,19 @@
     </row>
     <row r="46" spans="1:10" ht="105" x14ac:dyDescent="0.25">
       <c r="A46" s="11" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B46" s="11" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>124</v>
+        <v>274</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="F46" s="14">
         <v>2</v>
@@ -6744,19 +6744,19 @@
     </row>
     <row r="47" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A47" s="11" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B47" s="11" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="F47" s="14">
         <v>2</v>
@@ -6772,19 +6772,19 @@
     </row>
     <row r="48" spans="1:10" ht="120" x14ac:dyDescent="0.25">
       <c r="A48" s="11" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B48" s="11" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="F48" s="14">
         <v>2</v>
@@ -6800,19 +6800,19 @@
     </row>
     <row r="49" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="A49" s="11" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F49" s="14">
         <v>2</v>
@@ -6828,19 +6828,19 @@
     </row>
     <row r="50" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="11" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>130</v>
+        <v>273</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F50" s="14">
         <v>2</v>
@@ -6856,19 +6856,19 @@
     </row>
     <row r="51" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A51" s="12" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="B51" s="12" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="F51" s="14">
         <v>2</v>
@@ -6884,19 +6884,19 @@
     </row>
     <row r="52" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F52" s="14">
         <v>2</v>
@@ -6912,19 +6912,19 @@
     </row>
     <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="B53" s="12" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="F53" s="14">
         <v>2</v>
@@ -6940,19 +6940,19 @@
     </row>
     <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="12" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="B54" s="12" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>149</v>
+        <v>275</v>
       </c>
       <c r="F54" s="14">
         <v>2</v>
@@ -6968,19 +6968,19 @@
     </row>
     <row r="55" spans="1:10" ht="150" x14ac:dyDescent="0.25">
       <c r="A55" s="13" t="s">
-        <v>187</v>
+        <v>271</v>
       </c>
       <c r="B55" s="13" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="F55" s="14">
         <v>2</v>
@@ -6996,19 +6996,19 @@
     </row>
     <row r="56" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A56" s="13" t="s">
-        <v>187</v>
+        <v>271</v>
       </c>
       <c r="B56" s="13" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>253</v>
+        <v>269</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="F56" s="14">
         <v>2</v>
@@ -7024,19 +7024,19 @@
     </row>
     <row r="57" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A57" s="13" t="s">
-        <v>187</v>
+        <v>271</v>
       </c>
       <c r="B57" s="13" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="C57" s="19" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="E57" s="5" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="F57" s="14">
         <v>2</v>
@@ -7052,19 +7052,19 @@
     </row>
     <row r="58" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="13" t="s">
-        <v>187</v>
+        <v>271</v>
       </c>
       <c r="B58" s="13" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="E58" s="5" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="F58" s="14">
         <v>2</v>
@@ -7080,19 +7080,19 @@
     </row>
     <row r="59" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="13" t="s">
-        <v>187</v>
+        <v>271</v>
       </c>
       <c r="B59" s="13" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="E59" s="5" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="F59" s="14">
         <v>2</v>
@@ -7108,19 +7108,19 @@
     </row>
     <row r="60" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A60" s="13" t="s">
-        <v>187</v>
+        <v>271</v>
       </c>
       <c r="B60" s="13" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>168</v>
+        <v>268</v>
       </c>
       <c r="F60" s="14">
         <v>2</v>
@@ -7136,19 +7136,19 @@
     </row>
     <row r="61" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A61" s="13" t="s">
-        <v>187</v>
+        <v>271</v>
       </c>
       <c r="B61" s="13" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="F61" s="14">
         <v>2</v>
@@ -7206,18 +7206,18 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="B3" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C3" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -7343,7 +7343,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="B15">
         <v>2</v>
@@ -7354,7 +7354,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="B16">
         <v>24</v>
@@ -7429,7 +7429,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -7437,10 +7437,10 @@
         <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="C4" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fix: support quoted and multiline bulk question text import/export
- add a shared quote-aware question text parser
- support quoted, unquoted, and blank-line paragraph question formats
- preserve innapper quotes
- export round-trip-safe single-line er emphasis quotes while stripping legacy field wrquestion text records
- wire bulk actions and seeded question loading to the shared parser/formatter
- refresh reference question files, workbook source, and README guidance
- tighten gitignore and update app/server build artifacts
</commit_message>
<xml_diff>
--- a/data/ProjectMaturityAssessmentReviewTemplate.xlsx
+++ b/data/ProjectMaturityAssessmentReviewTemplate.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EE003AA-02EF-4B20-9201-346F02403F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C2BDC2F-8354-4A92-BF05-6FF9B636CB13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -924,9 +924,6 @@
     <t>Unstable test environments and data could increase the effort and lead to wrong results. For functional test and technical tests, test data management is an important prerequisite to ensure reasonable test results.</t>
   </si>
   <si>
-    <t>Support team needs good analysis options to solve incidents quickly to restore the ITservice as quickly as possible.</t>
-  </si>
-  <si>
     <t>This principle covers two aspects:
 •Deployable binaries of our software must always be build on a common build server (not on a developer machine)
 •Frequent builds ensure early feedback for timely corrective action if source code breaks
@@ -963,6 +960,9 @@
   </si>
   <si>
     <t>In order to supply robust and stable IT services we need to discuss disaster scenarios and mitigations with the business.</t>
+  </si>
+  <si>
+    <t>Support team needs good analysis options to solve incidents quickly to restore the IT service as quickly as possible.</t>
   </si>
 </sst>
 </file>
@@ -6049,7 +6049,7 @@
         <v>77</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>78</v>
@@ -6725,7 +6725,7 @@
         <v>122</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E46" s="5" t="s">
         <v>262</v>
@@ -6784,7 +6784,7 @@
         <v>126</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="F48" s="14">
         <v>2</v>
@@ -6834,7 +6834,7 @@
         <v>137</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>128</v>
@@ -6868,7 +6868,7 @@
         <v>139</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F51" s="14">
         <v>2</v>
@@ -6924,7 +6924,7 @@
         <v>143</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>264</v>
+        <v>275</v>
       </c>
       <c r="F53" s="14">
         <v>2</v>
@@ -6952,7 +6952,7 @@
         <v>145</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F54" s="14">
         <v>2</v>
@@ -6968,7 +6968,7 @@
     </row>
     <row r="55" spans="1:10" ht="150" x14ac:dyDescent="0.25">
       <c r="A55" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B55" s="13" t="s">
         <v>166</v>
@@ -6980,7 +6980,7 @@
         <v>246</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F55" s="14">
         <v>2</v>
@@ -6996,7 +6996,7 @@
     </row>
     <row r="56" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A56" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B56" s="13" t="s">
         <v>167</v>
@@ -7005,7 +7005,7 @@
         <v>151</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="E56" s="5" t="s">
         <v>152</v>
@@ -7024,7 +7024,7 @@
     </row>
     <row r="57" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A57" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B57" s="13" t="s">
         <v>168</v>
@@ -7052,7 +7052,7 @@
     </row>
     <row r="58" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B58" s="13" t="s">
         <v>169</v>
@@ -7080,7 +7080,7 @@
     </row>
     <row r="59" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B59" s="13" t="s">
         <v>170</v>
@@ -7108,7 +7108,7 @@
     </row>
     <row r="60" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A60" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B60" s="13" t="s">
         <v>171</v>
@@ -7120,7 +7120,7 @@
         <v>163</v>
       </c>
       <c r="E60" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="F60" s="14">
         <v>2</v>
@@ -7136,7 +7136,7 @@
     </row>
     <row r="61" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A61" s="13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B61" s="13" t="s">
         <v>172</v>
@@ -7148,7 +7148,7 @@
         <v>165</v>
       </c>
       <c r="E61" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F61" s="14">
         <v>2</v>

</xml_diff>